<commit_message>
Q1 2026 UPDATE - Enhanced coverage. Code2ISO.
</commit_message>
<xml_diff>
--- a/Excel-XLSX/UN-ANT.xlsx
+++ b/Excel-XLSX/UN-ANT.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>﻿"page"</t>
   </si>
@@ -63,106 +63,109 @@
     <t>asylum_seekers</t>
   </si>
   <si>
-    <t>returned_refugees</t>
-  </si>
-  <si>
     <t>idps</t>
   </si>
   <si>
-    <t>returned_idps</t>
+    <t>oip</t>
   </si>
   <si>
     <t>stateless</t>
   </si>
   <si>
+    <t>hst</t>
+  </si>
+  <si>
     <t>ooc</t>
   </si>
   <si>
-    <t>oip</t>
-  </si>
-  <si>
-    <t>hst</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
-    <t>jJG0k2</t>
-  </si>
-  <si>
-    <t>2007</t>
+    <t>C0Lpa7</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
+    <t>81</t>
+  </si>
+  <si>
+    <t>Haiti</t>
+  </si>
+  <si>
+    <t>HAI</t>
+  </si>
+  <si>
+    <t>HTI</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Antigua and Barbuda</t>
+  </si>
+  <si>
+    <t>ANT</t>
+  </si>
+  <si>
+    <t>ATG</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>115</t>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
-    <t>Afghanistan</t>
-  </si>
-  <si>
-    <t>AFG</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>Antigua and Barbuda</t>
-  </si>
-  <si>
-    <t>ANT</t>
-  </si>
-  <si>
-    <t>ATG</t>
-  </si>
-  <si>
-    <t>0</t>
+    <t>2015</t>
+  </si>
+  <si>
+    <t>185</t>
+  </si>
+  <si>
+    <t>Syrian Arab Rep.</t>
+  </si>
+  <si>
+    <t>SYR</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>2016</t>
   </si>
   <si>
     <t>5</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>2015</t>
-  </si>
-  <si>
-    <t>185</t>
-  </si>
-  <si>
-    <t>Syrian Arab Rep.</t>
-  </si>
-  <si>
-    <t>SYR</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>2016</t>
-  </si>
-  <si>
     <t>4</t>
   </si>
   <si>
-    <t>2022</t>
-  </si>
-  <si>
-    <t>81</t>
-  </si>
-  <si>
-    <t>Haiti</t>
-  </si>
-  <si>
-    <t>HAI</t>
-  </si>
-  <si>
-    <t>HTI</t>
-  </si>
-  <si>
-    <t>115</t>
+    <t>2024</t>
+  </si>
+  <si>
+    <t>203</t>
+  </si>
+  <si>
+    <t>Uzbekistan</t>
+  </si>
+  <si>
+    <t>UZB</t>
+  </si>
+  <si>
+    <t>2025</t>
+  </si>
+  <si>
+    <t>6</t>
   </si>
   <si>
     <t>207</t>
@@ -175,21 +178,6 @@
   </si>
   <si>
     <t>54</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>2024</t>
-  </si>
-  <si>
-    <t>203</t>
-  </si>
-  <si>
-    <t>Uzbekistan</t>
-  </si>
-  <si>
-    <t>UZB</t>
   </si>
 </sst>
 </file>
@@ -574,7 +562,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr defaultRowHeight="12.85"/>
   <sheetData>
     <row r="1">
@@ -638,93 +626,81 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>21</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="N2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="O2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="P2" s="2" t="s">
+      <c r="R2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="T2" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="R2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="S2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>35</v>
@@ -742,54 +718,48 @@
         <v>38</v>
       </c>
       <c r="J3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="N3" s="2" t="s">
         <v>39</v>
       </c>
       <c r="O3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="P3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="R3" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>40</v>
@@ -810,247 +780,223 @@
         <v>38</v>
       </c>
       <c r="J4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="M4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M4" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="N4" s="2" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="O4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="P4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q4" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="R4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="V4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>47</v>
       </c>
       <c r="J5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="L5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="M5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M5" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="N5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="O5" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="P5" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q5" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="R5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="V5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="J6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="M6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M6" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="N6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="O6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="P6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q6" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="R6" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="V6" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="F7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="R7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="T7" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="O7" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="P7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="R7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="S7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="T7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="V7" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>